<commit_message>
Move PLAYGROUP to CRECHE and update balances
Update class assignments and outstanding totals: docs/data/meta.json timestamp updated; PLAYGROUP 1 count decreased 21→18 and CRECHE added (3); currentOutstanding reduced by 123,870 to 7,759,440. In docs/data/students.json three students were moved from PLAYGROUP 1 to CRECHE, their latestBalance and 1st-term totals/balances reduced (each −41,290) and several fee line items simplified (NB & STAT set to 3050). Updated source/2026 - 2027 FEE.xlsx accordingly.
</commit_message>
<xml_diff>
--- a/source/2026 - 2027 FEE.xlsx
+++ b/source/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E74E945-2CD0-43F7-8B64-DC4CAD2F27EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9888DF-3D94-470D-B6B1-86121ACF596C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="254">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -797,6 +797,9 @@
   <si>
     <t>DAVID OLUWADARASIMI</t>
   </si>
+  <si>
+    <t>CRECHE</t>
+  </si>
 </sst>
 </file>
 
@@ -1419,13 +1422,13 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>34</v>
+        <v>143</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>197</v>
+        <v>241</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>36</v>
+        <v>253</v>
       </c>
       <c r="D2" s="16">
         <v>0.25</v>
@@ -1434,16 +1437,16 @@
         <v>0</v>
       </c>
       <c r="F2" s="17">
-        <v>33000</v>
+        <v>26000</v>
       </c>
       <c r="G2" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H2" s="17">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I2" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="J2" s="17">
         <f>(1-$D2)*E2</f>
@@ -1451,25 +1454,25 @@
       </c>
       <c r="K2" s="17">
         <f>(1-$D2)*F2</f>
-        <v>24750</v>
+        <v>19500</v>
       </c>
       <c r="L2" s="17">
         <f>G2</f>
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="M2" s="17">
         <f>(1-$D2)*H2</f>
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="N2" s="17">
         <f>(1-$D2)*I2</f>
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="O2" s="17">
-        <v>19560</v>
+        <v>0</v>
       </c>
       <c r="P2" s="17">
-        <v>14330</v>
+        <v>3050</v>
       </c>
       <c r="Q2" s="17">
         <v>0</v>
@@ -1481,7 +1484,7 @@
         <v>0</v>
       </c>
       <c r="T2" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="U2" s="17">
         <v>0</v>
@@ -1496,18 +1499,18 @@
         <v>0</v>
       </c>
       <c r="Y2" s="17">
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="17">
         <f>SUM(J2:Y2)</f>
-        <v>78390</v>
+        <v>27300</v>
       </c>
       <c r="AA2" s="17">
         <v>0</v>
       </c>
       <c r="AB2" s="14">
         <f>Z2-AA2</f>
-        <v>78390</v>
+        <v>27300</v>
       </c>
       <c r="AC2" s="17" t="str">
         <f>IF(AND($T2=6000, ($T2+$W2-$AB2)&gt;=6000),T2,"")</f>
@@ -1524,31 +1527,31 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>53</v>
+        <v>242</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>36</v>
+        <v>253</v>
       </c>
       <c r="D3" s="16">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E3" s="17">
         <v>0</v>
       </c>
       <c r="F3" s="17">
-        <v>33000</v>
+        <v>26000</v>
       </c>
       <c r="G3" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H3" s="17">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I3" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="J3" s="17">
         <f>(1-$D3)*E3</f>
@@ -1556,25 +1559,25 @@
       </c>
       <c r="K3" s="17">
         <f>(1-$D3)*F3</f>
-        <v>23100</v>
+        <v>26000</v>
       </c>
       <c r="L3" s="17">
         <f>G3</f>
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="M3" s="17">
         <f>(1-$D3)*H3</f>
-        <v>1400</v>
+        <v>1000</v>
       </c>
       <c r="N3" s="17">
         <f>(1-$D3)*I3</f>
-        <v>4200</v>
+        <v>0</v>
       </c>
       <c r="O3" s="17">
-        <v>19560</v>
+        <v>0</v>
       </c>
       <c r="P3" s="17">
-        <v>14330</v>
+        <v>3050</v>
       </c>
       <c r="Q3" s="17">
         <v>0</v>
@@ -1605,14 +1608,14 @@
       </c>
       <c r="Z3" s="17">
         <f>SUM(J3:Y3)</f>
-        <v>67590</v>
+        <v>34050</v>
       </c>
       <c r="AA3" s="17">
         <v>0</v>
       </c>
       <c r="AB3" s="14">
         <f>Z3-AA3</f>
-        <v>67590</v>
+        <v>34050</v>
       </c>
       <c r="AC3" s="17" t="str">
         <f>IF(AND($T3=6000, ($T3+$W3-$AB3)&gt;=6000),T3,"")</f>
@@ -1629,13 +1632,13 @@
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>57</v>
+        <v>121</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>179</v>
+        <v>243</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>36</v>
+        <v>253</v>
       </c>
       <c r="D4" s="16">
         <v>0.25</v>
@@ -1644,16 +1647,16 @@
         <v>0</v>
       </c>
       <c r="F4" s="17">
-        <v>33000</v>
+        <v>26000</v>
       </c>
       <c r="G4" s="17">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H4" s="17">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I4" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="J4" s="17">
         <f>(1-$D4)*E4</f>
@@ -1661,25 +1664,25 @@
       </c>
       <c r="K4" s="17">
         <f>(1-$D4)*F4</f>
-        <v>24750</v>
+        <v>19500</v>
       </c>
       <c r="L4" s="17">
         <f>G4</f>
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="M4" s="17">
         <f>(1-$D4)*H4</f>
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="N4" s="17">
         <f>(1-$D4)*I4</f>
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="O4" s="17">
-        <v>19560</v>
+        <v>0</v>
       </c>
       <c r="P4" s="17">
-        <v>14330</v>
+        <v>3050</v>
       </c>
       <c r="Q4" s="17">
         <v>0</v>
@@ -1710,14 +1713,14 @@
       </c>
       <c r="Z4" s="17">
         <f>SUM(J4:Y4)</f>
-        <v>69640</v>
+        <v>27300</v>
       </c>
       <c r="AA4" s="17">
         <v>0</v>
       </c>
       <c r="AB4" s="14">
         <f>Z4-AA4</f>
-        <v>69640</v>
+        <v>27300</v>
       </c>
       <c r="AC4" s="17" t="str">
         <f>IF(AND($T4=6000, ($T4+$W4-$AB4)&gt;=6000),T4,"")</f>
@@ -1734,16 +1737,16 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>195</v>
+        <v>34</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>36</v>
       </c>
       <c r="D5" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E5" s="17">
         <v>0</v>
@@ -1766,7 +1769,7 @@
       </c>
       <c r="K5" s="17">
         <f>(1-$D5)*F5</f>
-        <v>33000</v>
+        <v>24750</v>
       </c>
       <c r="L5" s="17">
         <f>G5</f>
@@ -1774,11 +1777,11 @@
       </c>
       <c r="M5" s="17">
         <f>(1-$D5)*H5</f>
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="N5" s="17">
         <f>(1-$D5)*I5</f>
-        <v>6000</v>
+        <v>4500</v>
       </c>
       <c r="O5" s="17">
         <v>19560</v>
@@ -1796,7 +1799,7 @@
         <v>0</v>
       </c>
       <c r="T5" s="17">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="U5" s="17">
         <v>0</v>
@@ -1811,18 +1814,18 @@
         <v>0</v>
       </c>
       <c r="Y5" s="17">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="Z5" s="17">
         <f>SUM(J5:Y5)</f>
-        <v>79890</v>
+        <v>78390</v>
       </c>
       <c r="AA5" s="17">
         <v>0</v>
       </c>
       <c r="AB5" s="14">
         <f>Z5-AA5</f>
-        <v>79890</v>
+        <v>78390</v>
       </c>
       <c r="AC5" s="17" t="str">
         <f>IF(AND($T5=6000, ($T5+$W5-$AB5)&gt;=6000),T5,"")</f>
@@ -1839,10 +1842,10 @@
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>36</v>
@@ -1944,16 +1947,16 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>51</v>
+        <v>179</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D7" s="16">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="E7" s="17">
         <v>0</v>
@@ -1976,7 +1979,7 @@
       </c>
       <c r="K7" s="17">
         <f>(1-$D7)*F7</f>
-        <v>16500</v>
+        <v>24750</v>
       </c>
       <c r="L7" s="17">
         <f>G7</f>
@@ -1984,14 +1987,14 @@
       </c>
       <c r="M7" s="17">
         <f>(1-$D7)*H7</f>
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="N7" s="17">
         <f>(1-$D7)*I7</f>
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="O7" s="17">
-        <v>22580</v>
+        <v>19560</v>
       </c>
       <c r="P7" s="17">
         <v>14330</v>
@@ -2025,14 +2028,14 @@
       </c>
       <c r="Z7" s="17">
         <f>SUM(J7:Y7)</f>
-        <v>62410</v>
+        <v>69640</v>
       </c>
       <c r="AA7" s="17">
         <v>0</v>
       </c>
       <c r="AB7" s="14">
         <f>Z7-AA7</f>
-        <v>62410</v>
+        <v>69640</v>
       </c>
       <c r="AC7" s="17" t="str">
         <f>IF(AND($T7=6000, ($T7+$W7-$AB7)&gt;=6000),T7,"")</f>
@@ -2049,16 +2052,16 @@
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>57</v>
+        <v>195</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>58</v>
+        <v>196</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D8" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E8" s="17">
         <v>0</v>
@@ -2081,7 +2084,7 @@
       </c>
       <c r="K8" s="17">
         <f>(1-$D8)*F8</f>
-        <v>16500</v>
+        <v>33000</v>
       </c>
       <c r="L8" s="17">
         <f>G8</f>
@@ -2089,14 +2092,14 @@
       </c>
       <c r="M8" s="17">
         <f>(1-$D8)*H8</f>
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="N8" s="17">
         <f>(1-$D8)*I8</f>
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="O8" s="17">
-        <v>22580</v>
+        <v>19560</v>
       </c>
       <c r="P8" s="17">
         <v>14330</v>
@@ -2130,14 +2133,14 @@
       </c>
       <c r="Z8" s="17">
         <f>SUM(J8:Y8)</f>
-        <v>62410</v>
+        <v>79890</v>
       </c>
       <c r="AA8" s="17">
         <v>0</v>
       </c>
       <c r="AB8" s="14">
         <f>Z8-AA8</f>
-        <v>62410</v>
+        <v>79890</v>
       </c>
       <c r="AC8" s="17" t="str">
         <f>IF(AND($T8=6000, ($T8+$W8-$AB8)&gt;=6000),T8,"")</f>
@@ -2154,16 +2157,16 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D9" s="16">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E9" s="17">
         <v>0</v>
@@ -2186,7 +2189,7 @@
       </c>
       <c r="K9" s="17">
         <f>(1-$D9)*F9</f>
-        <v>16500</v>
+        <v>23100</v>
       </c>
       <c r="L9" s="17">
         <f>G9</f>
@@ -2194,14 +2197,14 @@
       </c>
       <c r="M9" s="17">
         <f>(1-$D9)*H9</f>
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="N9" s="17">
         <f>(1-$D9)*I9</f>
-        <v>3000</v>
+        <v>4200</v>
       </c>
       <c r="O9" s="17">
-        <v>22580</v>
+        <v>19560</v>
       </c>
       <c r="P9" s="17">
         <v>14330</v>
@@ -2216,7 +2219,7 @@
         <v>0</v>
       </c>
       <c r="T9" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="U9" s="17">
         <v>0</v>
@@ -2231,18 +2234,18 @@
         <v>0</v>
       </c>
       <c r="Y9" s="17">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="17">
         <f>SUM(J9:Y9)</f>
-        <v>70380</v>
+        <v>67590</v>
       </c>
       <c r="AA9" s="17">
         <v>0</v>
       </c>
       <c r="AB9" s="14">
         <f>Z9-AA9</f>
-        <v>70380</v>
+        <v>67590</v>
       </c>
       <c r="AC9" s="17" t="str">
         <f>IF(AND($T9=6000, ($T9+$W9-$AB9)&gt;=6000),T9,"")</f>
@@ -2259,16 +2262,16 @@
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>67</v>
       </c>
       <c r="D10" s="16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="17">
         <v>0</v>
@@ -2291,7 +2294,7 @@
       </c>
       <c r="K10" s="17">
         <f>(1-$D10)*F10</f>
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="L10" s="17">
         <f>G10</f>
@@ -2299,11 +2302,11 @@
       </c>
       <c r="M10" s="17">
         <f>(1-$D10)*H10</f>
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="N10" s="17">
         <f>(1-$D10)*I10</f>
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="O10" s="17">
         <v>22580</v>
@@ -2336,18 +2339,18 @@
         <v>0</v>
       </c>
       <c r="Y10" s="17">
-        <v>-8970</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="17">
         <f>SUM(J10:Y10)</f>
-        <v>73940</v>
+        <v>62410</v>
       </c>
       <c r="AA10" s="17">
         <v>0</v>
       </c>
       <c r="AB10" s="14">
         <f>Z10-AA10</f>
-        <v>73940</v>
+        <v>62410</v>
       </c>
       <c r="AC10" s="17" t="str">
         <f>IF(AND($T10=6000, ($T10+$W10-$AB10)&gt;=6000),T10,"")</f>
@@ -2364,10 +2367,10 @@
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>67</v>
@@ -2441,18 +2444,18 @@
         <v>0</v>
       </c>
       <c r="Y11" s="17">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="17">
         <f>SUM(J11:Y11)</f>
-        <v>62890</v>
+        <v>62410</v>
       </c>
       <c r="AA11" s="17">
         <v>0</v>
       </c>
       <c r="AB11" s="14">
         <f>Z11-AA11</f>
-        <v>62890</v>
+        <v>62410</v>
       </c>
       <c r="AC11" s="17" t="str">
         <f>IF(AND($T11=6000, ($T11+$W11-$AB11)&gt;=6000),T11,"")</f>
@@ -2469,16 +2472,16 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>191</v>
+        <v>65</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>199</v>
+        <v>66</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="16">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="17">
         <v>0</v>
@@ -2501,7 +2504,7 @@
       </c>
       <c r="K12" s="17">
         <f>(1-$D12)*F12</f>
-        <v>24750</v>
+        <v>16500</v>
       </c>
       <c r="L12" s="17">
         <f>G12</f>
@@ -2509,11 +2512,11 @@
       </c>
       <c r="M12" s="17">
         <f>(1-$D12)*H12</f>
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="N12" s="17">
         <f>(1-$D12)*I12</f>
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="O12" s="17">
         <v>22580</v>
@@ -2531,7 +2534,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="17">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="U12" s="17">
         <v>0</v>
@@ -2546,18 +2549,18 @@
         <v>0</v>
       </c>
       <c r="Y12" s="17">
-        <v>0</v>
+        <v>-30</v>
       </c>
       <c r="Z12" s="17">
         <f>SUM(J12:Y12)</f>
-        <v>72660</v>
+        <v>70380</v>
       </c>
       <c r="AA12" s="17">
         <v>0</v>
       </c>
       <c r="AB12" s="14">
         <f>Z12-AA12</f>
-        <v>72660</v>
+        <v>70380</v>
       </c>
       <c r="AC12" s="17" t="str">
         <f>IF(AND($T12=6000, ($T12+$W12-$AB12)&gt;=6000),T12,"")</f>
@@ -2574,16 +2577,16 @@
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>67</v>
       </c>
       <c r="D13" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E13" s="17">
         <v>0</v>
@@ -2606,7 +2609,7 @@
       </c>
       <c r="K13" s="17">
         <f>(1-$D13)*F13</f>
-        <v>16500</v>
+        <v>33000</v>
       </c>
       <c r="L13" s="17">
         <f>G13</f>
@@ -2614,11 +2617,11 @@
       </c>
       <c r="M13" s="17">
         <f>(1-$D13)*H13</f>
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="N13" s="17">
         <f>(1-$D13)*I13</f>
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="O13" s="17">
         <v>22580</v>
@@ -2651,18 +2654,18 @@
         <v>0</v>
       </c>
       <c r="Y13" s="17">
-        <v>500</v>
+        <v>-8970</v>
       </c>
       <c r="Z13" s="17">
         <f>SUM(J13:Y13)</f>
-        <v>62910</v>
+        <v>73940</v>
       </c>
       <c r="AA13" s="17">
         <v>0</v>
       </c>
       <c r="AB13" s="14">
         <f>Z13-AA13</f>
-        <v>62910</v>
+        <v>73940</v>
       </c>
       <c r="AC13" s="17" t="str">
         <f>IF(AND($T13=6000, ($T13+$W13-$AB13)&gt;=6000),T13,"")</f>
@@ -2679,10 +2682,10 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>67</v>
@@ -2756,18 +2759,18 @@
         <v>0</v>
       </c>
       <c r="Y14" s="17">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="Z14" s="17">
         <f>SUM(J14:Y14)</f>
-        <v>62410</v>
+        <v>62890</v>
       </c>
       <c r="AA14" s="17">
         <v>0</v>
       </c>
       <c r="AB14" s="14">
         <f>Z14-AA14</f>
-        <v>62410</v>
+        <v>62890</v>
       </c>
       <c r="AC14" s="17" t="str">
         <f>IF(AND($T14=6000, ($T14+$W14-$AB14)&gt;=6000),T14,"")</f>
@@ -2784,16 +2787,16 @@
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>111</v>
+        <v>191</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>112</v>
+        <v>199</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>67</v>
       </c>
       <c r="D15" s="16">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="E15" s="17">
         <v>0</v>
@@ -2816,7 +2819,7 @@
       </c>
       <c r="K15" s="17">
         <f>(1-$D15)*F15</f>
-        <v>23100</v>
+        <v>24750</v>
       </c>
       <c r="L15" s="17">
         <f>G15</f>
@@ -2824,11 +2827,11 @@
       </c>
       <c r="M15" s="17">
         <f>(1-$D15)*H15</f>
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="N15" s="17">
         <f>(1-$D15)*I15</f>
-        <v>4200</v>
+        <v>4500</v>
       </c>
       <c r="O15" s="17">
         <v>22580</v>
@@ -2865,14 +2868,14 @@
       </c>
       <c r="Z15" s="17">
         <f>SUM(J15:Y15)</f>
-        <v>70610</v>
+        <v>72660</v>
       </c>
       <c r="AA15" s="17">
         <v>0</v>
       </c>
       <c r="AB15" s="14">
         <f>Z15-AA15</f>
-        <v>70610</v>
+        <v>72660</v>
       </c>
       <c r="AC15" s="17" t="str">
         <f>IF(AND($T15=6000, ($T15+$W15-$AB15)&gt;=6000),T15,"")</f>
@@ -2889,10 +2892,10 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>116</v>
+        <v>55</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>67</v>
@@ -2951,7 +2954,7 @@
         <v>0</v>
       </c>
       <c r="T16" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="U16" s="17">
         <v>0</v>
@@ -2966,18 +2969,18 @@
         <v>0</v>
       </c>
       <c r="Y16" s="17">
-        <v>-3145</v>
+        <v>500</v>
       </c>
       <c r="Z16" s="17">
         <f>SUM(J16:Y16)</f>
-        <v>67265</v>
+        <v>62910</v>
       </c>
       <c r="AA16" s="17">
         <v>0</v>
       </c>
       <c r="AB16" s="14">
         <f>Z16-AA16</f>
-        <v>67265</v>
+        <v>62910</v>
       </c>
       <c r="AC16" s="17" t="str">
         <f>IF(AND($T16=6000, ($T16+$W16-$AB16)&gt;=6000),T16,"")</f>
@@ -2994,16 +2997,16 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="C17" s="15" t="s">
         <v>67</v>
       </c>
       <c r="D17" s="16">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="17">
         <v>0</v>
@@ -3026,7 +3029,7 @@
       </c>
       <c r="K17" s="17">
         <f>(1-$D17)*F17</f>
-        <v>23100</v>
+        <v>16500</v>
       </c>
       <c r="L17" s="17">
         <f>G17</f>
@@ -3034,11 +3037,11 @@
       </c>
       <c r="M17" s="17">
         <f>(1-$D17)*H17</f>
-        <v>1400</v>
+        <v>1000</v>
       </c>
       <c r="N17" s="17">
         <f>(1-$D17)*I17</f>
-        <v>4200</v>
+        <v>3000</v>
       </c>
       <c r="O17" s="17">
         <v>22580</v>
@@ -3056,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="T17" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="U17" s="17">
         <v>0</v>
@@ -3075,14 +3078,14 @@
       </c>
       <c r="Z17" s="17">
         <f>SUM(J17:Y17)</f>
-        <v>78610</v>
+        <v>62410</v>
       </c>
       <c r="AA17" s="17">
         <v>0</v>
       </c>
       <c r="AB17" s="14">
         <f>Z17-AA17</f>
-        <v>78610</v>
+        <v>62410</v>
       </c>
       <c r="AC17" s="17" t="str">
         <f>IF(AND($T17=6000, ($T17+$W17-$AB17)&gt;=6000),T17,"")</f>
@@ -3099,31 +3102,31 @@
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>236</v>
+        <v>111</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>240</v>
+        <v>112</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D18" s="16">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E18" s="17">
         <v>0</v>
       </c>
       <c r="F18" s="17">
-        <v>26000</v>
+        <v>33000</v>
       </c>
       <c r="G18" s="17">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="H18" s="17">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I18" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J18" s="17">
         <f>(1-$D18)*E18</f>
@@ -3131,25 +3134,25 @@
       </c>
       <c r="K18" s="17">
         <f>(1-$D18)*F18</f>
-        <v>19500</v>
+        <v>23100</v>
       </c>
       <c r="L18" s="17">
         <f>G18</f>
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="M18" s="17">
         <f>(1-$D18)*H18</f>
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="N18" s="17">
         <f>(1-$D18)*I18</f>
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="O18" s="17">
-        <v>13080</v>
+        <v>22580</v>
       </c>
       <c r="P18" s="17">
-        <v>7550</v>
+        <v>14330</v>
       </c>
       <c r="Q18" s="17">
         <v>0</v>
@@ -3161,7 +3164,7 @@
         <v>0</v>
       </c>
       <c r="T18" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U18" s="17">
         <v>0</v>
@@ -3176,18 +3179,18 @@
         <v>0</v>
       </c>
       <c r="Y18" s="17">
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="17">
         <f>SUM(J18:Y18)</f>
-        <v>50880</v>
+        <v>70610</v>
       </c>
       <c r="AA18" s="17">
         <v>0</v>
       </c>
       <c r="AB18" s="14">
         <f>Z18-AA18</f>
-        <v>50880</v>
+        <v>70610</v>
       </c>
       <c r="AC18" s="17" t="str">
         <f>IF(AND($T18=6000, ($T18+$W18-$AB18)&gt;=6000),T18,"")</f>
@@ -3204,31 +3207,31 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>182</v>
+        <v>116</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>209</v>
+        <v>117</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D19" s="16">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E19" s="17">
         <v>0</v>
       </c>
       <c r="F19" s="17">
-        <v>26000</v>
+        <v>33000</v>
       </c>
       <c r="G19" s="17">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="H19" s="17">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I19" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J19" s="17">
         <f>(1-$D19)*E19</f>
@@ -3236,25 +3239,25 @@
       </c>
       <c r="K19" s="17">
         <f>(1-$D19)*F19</f>
-        <v>19500</v>
+        <v>16500</v>
       </c>
       <c r="L19" s="17">
         <f>G19</f>
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="M19" s="17">
         <f>(1-$D19)*H19</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="N19" s="17">
         <f>(1-$D19)*I19</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="O19" s="17">
-        <v>13080</v>
+        <v>22580</v>
       </c>
       <c r="P19" s="17">
-        <v>7550</v>
+        <v>14330</v>
       </c>
       <c r="Q19" s="17">
         <v>0</v>
@@ -3266,7 +3269,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="17">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="U19" s="17">
         <v>0</v>
@@ -3281,18 +3284,18 @@
         <v>0</v>
       </c>
       <c r="Y19" s="17">
-        <v>0</v>
+        <v>-3145</v>
       </c>
       <c r="Z19" s="17">
         <f>SUM(J19:Y19)</f>
-        <v>44130</v>
+        <v>67265</v>
       </c>
       <c r="AA19" s="17">
         <v>0</v>
       </c>
       <c r="AB19" s="14">
         <f>Z19-AA19</f>
-        <v>44130</v>
+        <v>67265</v>
       </c>
       <c r="AC19" s="17" t="str">
         <f>IF(AND($T19=6000, ($T19+$W19-$AB19)&gt;=6000),T19,"")</f>
@@ -3309,31 +3312,31 @@
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D20" s="16">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E20" s="17">
         <v>0</v>
       </c>
       <c r="F20" s="17">
-        <v>26000</v>
+        <v>33000</v>
       </c>
       <c r="G20" s="17">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="H20" s="17">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I20" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J20" s="17">
         <f>(1-$D20)*E20</f>
@@ -3341,25 +3344,25 @@
       </c>
       <c r="K20" s="17">
         <f>(1-$D20)*F20</f>
-        <v>19500</v>
+        <v>23100</v>
       </c>
       <c r="L20" s="17">
         <f>G20</f>
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="M20" s="17">
         <f>(1-$D20)*H20</f>
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="N20" s="17">
         <f>(1-$D20)*I20</f>
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="O20" s="17">
-        <v>13080</v>
+        <v>22580</v>
       </c>
       <c r="P20" s="17">
-        <v>7550</v>
+        <v>14330</v>
       </c>
       <c r="Q20" s="17">
         <v>0</v>
@@ -3371,7 +3374,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="17">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="U20" s="17">
         <v>0</v>
@@ -3390,14 +3393,14 @@
       </c>
       <c r="Z20" s="17">
         <f>SUM(J20:Y20)</f>
-        <v>50130</v>
+        <v>78610</v>
       </c>
       <c r="AA20" s="17">
         <v>0</v>
       </c>
       <c r="AB20" s="14">
         <f>Z20-AA20</f>
-        <v>50130</v>
+        <v>78610</v>
       </c>
       <c r="AC20" s="17" t="str">
         <f>IF(AND($T20=6000, ($T20+$W20-$AB20)&gt;=6000),T20,"")</f>
@@ -3414,16 +3417,16 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>63</v>
+        <v>236</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>54</v>
+        <v>240</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D21" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E21" s="17">
         <v>0</v>
@@ -3446,7 +3449,7 @@
       </c>
       <c r="K21" s="17">
         <f>(1-$D21)*F21</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L21" s="17">
         <f>G21</f>
@@ -3491,18 +3494,18 @@
         <v>0</v>
       </c>
       <c r="Y21" s="17">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="Z21" s="17">
         <f>SUM(J21:Y21)</f>
-        <v>56630</v>
+        <v>50880</v>
       </c>
       <c r="AA21" s="17">
         <v>0</v>
       </c>
       <c r="AB21" s="14">
         <f>Z21-AA21</f>
-        <v>56630</v>
+        <v>50880</v>
       </c>
       <c r="AC21" s="17" t="str">
         <f>IF(AND($T21=6000, ($T21+$W21-$AB21)&gt;=6000),T21,"")</f>
@@ -3519,16 +3522,16 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>156</v>
+        <v>209</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D22" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E22" s="17">
         <v>0</v>
@@ -3551,7 +3554,7 @@
       </c>
       <c r="K22" s="17">
         <f>(1-$D22)*F22</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L22" s="17">
         <f>G22</f>
@@ -3581,7 +3584,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U22" s="17">
         <v>0</v>
@@ -3600,14 +3603,14 @@
       </c>
       <c r="Z22" s="17">
         <f>SUM(J22:Y22)</f>
-        <v>56630</v>
+        <v>44130</v>
       </c>
       <c r="AA22" s="17">
         <v>0</v>
       </c>
       <c r="AB22" s="14">
         <f>Z22-AA22</f>
-        <v>56630</v>
+        <v>44130</v>
       </c>
       <c r="AC22" s="17" t="str">
         <f>IF(AND($T22=6000, ($T22+$W22-$AB22)&gt;=6000),T22,"")</f>
@@ -3624,16 +3627,16 @@
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D23" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E23" s="17">
         <v>0</v>
@@ -3656,7 +3659,7 @@
       </c>
       <c r="K23" s="17">
         <f>(1-$D23)*F23</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L23" s="17">
         <f>G23</f>
@@ -3686,7 +3689,7 @@
         <v>0</v>
       </c>
       <c r="T23" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U23" s="17">
         <v>0</v>
@@ -3705,14 +3708,14 @@
       </c>
       <c r="Z23" s="17">
         <f>SUM(J23:Y23)</f>
-        <v>50630</v>
+        <v>50130</v>
       </c>
       <c r="AA23" s="17">
         <v>0</v>
       </c>
       <c r="AB23" s="14">
         <f>Z23-AA23</f>
-        <v>50630</v>
+        <v>50130</v>
       </c>
       <c r="AC23" s="17" t="str">
         <f>IF(AND($T23=6000, ($T23+$W23-$AB23)&gt;=6000),T23,"")</f>
@@ -3729,10 +3732,10 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>235</v>
+        <v>54</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>44</v>
@@ -3806,18 +3809,18 @@
         <v>0</v>
       </c>
       <c r="Y24" s="17">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="Z24" s="17">
         <f>SUM(J24:Y24)</f>
-        <v>57630</v>
+        <v>56630</v>
       </c>
       <c r="AA24" s="17">
         <v>0</v>
       </c>
       <c r="AB24" s="14">
         <f>Z24-AA24</f>
-        <v>57630</v>
+        <v>56630</v>
       </c>
       <c r="AC24" s="17" t="str">
         <f>IF(AND($T24=6000, ($T24+$W24-$AB24)&gt;=6000),T24,"")</f>
@@ -3834,16 +3837,16 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>73</v>
+        <v>156</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D25" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E25" s="17">
         <v>0</v>
@@ -3866,7 +3869,7 @@
       </c>
       <c r="K25" s="17">
         <f>(1-$D25)*F25</f>
-        <v>13000</v>
+        <v>26000</v>
       </c>
       <c r="L25" s="17">
         <f>G25</f>
@@ -3896,7 +3899,7 @@
         <v>0</v>
       </c>
       <c r="T25" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U25" s="17">
         <v>0</v>
@@ -3911,18 +3914,18 @@
         <v>0</v>
       </c>
       <c r="Y25" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="Z25" s="17">
         <f>SUM(J25:Y25)</f>
-        <v>45630</v>
+        <v>56630</v>
       </c>
       <c r="AA25" s="17">
         <v>0</v>
       </c>
       <c r="AB25" s="14">
         <f>Z25-AA25</f>
-        <v>45630</v>
+        <v>56630</v>
       </c>
       <c r="AC25" s="17" t="str">
         <f>IF(AND($T25=6000, ($T25+$W25-$AB25)&gt;=6000),T25,"")</f>
@@ -3939,16 +3942,16 @@
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D26" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E26" s="17">
         <v>0</v>
@@ -3971,7 +3974,7 @@
       </c>
       <c r="K26" s="17">
         <f>(1-$D26)*F26</f>
-        <v>13000</v>
+        <v>26000</v>
       </c>
       <c r="L26" s="17">
         <f>G26</f>
@@ -4016,18 +4019,18 @@
         <v>0</v>
       </c>
       <c r="Y26" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="Z26" s="17">
         <f>SUM(J26:Y26)</f>
-        <v>45630</v>
+        <v>50630</v>
       </c>
       <c r="AA26" s="17">
         <v>0</v>
       </c>
       <c r="AB26" s="14">
         <f>Z26-AA26</f>
-        <v>45630</v>
+        <v>50630</v>
       </c>
       <c r="AC26" s="17" t="str">
         <f>IF(AND($T26=6000, ($T26+$W26-$AB26)&gt;=6000),T26,"")</f>
@@ -4044,16 +4047,16 @@
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>159</v>
+        <v>234</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>160</v>
+        <v>235</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D27" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E27" s="17">
         <v>0</v>
@@ -4076,7 +4079,7 @@
       </c>
       <c r="K27" s="17">
         <f>(1-$D27)*F27</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L27" s="17">
         <f>G27</f>
@@ -4121,18 +4124,18 @@
         <v>0</v>
       </c>
       <c r="Y27" s="17">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="Z27" s="17">
         <f>SUM(J27:Y27)</f>
-        <v>50130</v>
+        <v>57630</v>
       </c>
       <c r="AA27" s="17">
         <v>0</v>
       </c>
       <c r="AB27" s="14">
         <f>Z27-AA27</f>
-        <v>50130</v>
+        <v>57630</v>
       </c>
       <c r="AC27" s="17" t="str">
         <f>IF(AND($T27=6000, ($T27+$W27-$AB27)&gt;=6000),T27,"")</f>
@@ -4149,16 +4152,16 @@
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D28" s="16">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E28" s="17">
         <v>0</v>
@@ -4181,7 +4184,7 @@
       </c>
       <c r="K28" s="17">
         <f>(1-$D28)*F28</f>
-        <v>19500</v>
+        <v>13000</v>
       </c>
       <c r="L28" s="17">
         <f>G28</f>
@@ -4211,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U28" s="17">
         <v>0</v>
@@ -4226,18 +4229,18 @@
         <v>0</v>
       </c>
       <c r="Y28" s="17">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="Z28" s="17">
         <f>SUM(J28:Y28)</f>
-        <v>50130</v>
+        <v>45630</v>
       </c>
       <c r="AA28" s="17">
         <v>0</v>
       </c>
       <c r="AB28" s="14">
         <f>Z28-AA28</f>
-        <v>50130</v>
+        <v>45630</v>
       </c>
       <c r="AC28" s="17" t="str">
         <f>IF(AND($T28=6000, ($T28+$W28-$AB28)&gt;=6000),T28,"")</f>
@@ -4254,16 +4257,16 @@
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>238</v>
+        <v>157</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>239</v>
+        <v>158</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D29" s="16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E29" s="17">
         <v>0</v>
@@ -4286,7 +4289,7 @@
       </c>
       <c r="K29" s="17">
         <f>(1-$D29)*F29</f>
-        <v>26000</v>
+        <v>13000</v>
       </c>
       <c r="L29" s="17">
         <f>G29</f>
@@ -4331,18 +4334,18 @@
         <v>0</v>
       </c>
       <c r="Y29" s="17">
-        <v>14000</v>
+        <v>8000</v>
       </c>
       <c r="Z29" s="17">
         <f>SUM(J29:Y29)</f>
-        <v>64630</v>
+        <v>45630</v>
       </c>
       <c r="AA29" s="17">
         <v>0</v>
       </c>
       <c r="AB29" s="14">
         <f>Z29-AA29</f>
-        <v>64630</v>
+        <v>45630</v>
       </c>
       <c r="AC29" s="17" t="str">
         <f>IF(AND($T29=6000, ($T29+$W29-$AB29)&gt;=6000),T29,"")</f>
@@ -4359,16 +4362,16 @@
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>93</v>
+        <v>159</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>94</v>
+        <v>160</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D30" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E30" s="17">
         <v>0</v>
@@ -4391,7 +4394,7 @@
       </c>
       <c r="K30" s="17">
         <f>(1-$D30)*F30</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L30" s="17">
         <f>G30</f>
@@ -4421,7 +4424,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U30" s="17">
         <v>0</v>
@@ -4436,18 +4439,18 @@
         <v>0</v>
       </c>
       <c r="Y30" s="17">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="Z30" s="17">
         <f>SUM(J30:Y30)</f>
-        <v>57630</v>
+        <v>50130</v>
       </c>
       <c r="AA30" s="17">
         <v>0</v>
       </c>
       <c r="AB30" s="14">
         <f>Z30-AA30</f>
-        <v>57630</v>
+        <v>50130</v>
       </c>
       <c r="AC30" s="17" t="str">
         <f>IF(AND($T30=6000, ($T30+$W30-$AB30)&gt;=6000),T30,"")</f>
@@ -4464,16 +4467,16 @@
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>100</v>
+        <v>161</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>101</v>
+        <v>163</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D31" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E31" s="17">
         <v>0</v>
@@ -4496,7 +4499,7 @@
       </c>
       <c r="K31" s="17">
         <f>(1-$D31)*F31</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L31" s="17">
         <f>G31</f>
@@ -4526,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U31" s="17">
         <v>0</v>
@@ -4541,18 +4544,18 @@
         <v>0</v>
       </c>
       <c r="Y31" s="17">
-        <v>-3030</v>
+        <v>0</v>
       </c>
       <c r="Z31" s="17">
         <f>SUM(J31:Y31)</f>
-        <v>47600</v>
+        <v>50130</v>
       </c>
       <c r="AA31" s="17">
         <v>0</v>
       </c>
       <c r="AB31" s="14">
         <f>Z31-AA31</f>
-        <v>47600</v>
+        <v>50130</v>
       </c>
       <c r="AC31" s="17" t="str">
         <f>IF(AND($T31=6000, ($T31+$W31-$AB31)&gt;=6000),T31,"")</f>
@@ -4569,10 +4572,10 @@
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>146</v>
+        <v>238</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>147</v>
+        <v>239</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>44</v>
@@ -4631,7 +4634,7 @@
         <v>0</v>
       </c>
       <c r="T32" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U32" s="17">
         <v>0</v>
@@ -4646,18 +4649,18 @@
         <v>0</v>
       </c>
       <c r="Y32" s="17">
-        <v>0</v>
+        <v>14000</v>
       </c>
       <c r="Z32" s="17">
         <f>SUM(J32:Y32)</f>
-        <v>56630</v>
+        <v>64630</v>
       </c>
       <c r="AA32" s="17">
         <v>0</v>
       </c>
       <c r="AB32" s="14">
         <f>Z32-AA32</f>
-        <v>56630</v>
+        <v>64630</v>
       </c>
       <c r="AC32" s="17" t="str">
         <f>IF(AND($T32=6000, ($T32+$W32-$AB32)&gt;=6000),T32,"")</f>
@@ -4674,16 +4677,16 @@
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D33" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E33" s="17">
         <v>0</v>
@@ -4706,7 +4709,7 @@
       </c>
       <c r="K33" s="17">
         <f>(1-$D33)*F33</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L33" s="17">
         <f>G33</f>
@@ -4736,7 +4739,7 @@
         <v>0</v>
       </c>
       <c r="T33" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U33" s="17">
         <v>0</v>
@@ -4751,18 +4754,18 @@
         <v>0</v>
       </c>
       <c r="Y33" s="17">
-        <v>0</v>
+        <v>7000</v>
       </c>
       <c r="Z33" s="17">
         <f>SUM(J33:Y33)</f>
-        <v>50130</v>
+        <v>57630</v>
       </c>
       <c r="AA33" s="17">
         <v>0</v>
       </c>
       <c r="AB33" s="14">
         <f>Z33-AA33</f>
-        <v>50130</v>
+        <v>57630</v>
       </c>
       <c r="AC33" s="17" t="str">
         <f>IF(AND($T33=6000, ($T33+$W33-$AB33)&gt;=6000),T33,"")</f>
@@ -4779,16 +4782,16 @@
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D34" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E34" s="17">
         <v>0</v>
@@ -4811,7 +4814,7 @@
       </c>
       <c r="K34" s="17">
         <f>(1-$D34)*F34</f>
-        <v>13000</v>
+        <v>26000</v>
       </c>
       <c r="L34" s="17">
         <f>G34</f>
@@ -4856,18 +4859,18 @@
         <v>0</v>
       </c>
       <c r="Y34" s="17">
-        <v>8000</v>
+        <v>-3030</v>
       </c>
       <c r="Z34" s="17">
         <f>SUM(J34:Y34)</f>
-        <v>45630</v>
+        <v>47600</v>
       </c>
       <c r="AA34" s="17">
         <v>0</v>
       </c>
       <c r="AB34" s="14">
         <f>Z34-AA34</f>
-        <v>45630</v>
+        <v>47600</v>
       </c>
       <c r="AC34" s="17" t="str">
         <f>IF(AND($T34=6000, ($T34+$W34-$AB34)&gt;=6000),T34,"")</f>
@@ -4884,16 +4887,16 @@
     </row>
     <row r="35" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D35" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E35" s="17">
         <v>0</v>
@@ -4916,7 +4919,7 @@
       </c>
       <c r="K35" s="17">
         <f>(1-$D35)*F35</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L35" s="17">
         <f>G35</f>
@@ -4946,7 +4949,7 @@
         <v>0</v>
       </c>
       <c r="T35" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U35" s="17">
         <v>0</v>
@@ -4965,14 +4968,14 @@
       </c>
       <c r="Z35" s="17">
         <f>SUM(J35:Y35)</f>
-        <v>44130</v>
+        <v>56630</v>
       </c>
       <c r="AA35" s="17">
         <v>0</v>
       </c>
       <c r="AB35" s="14">
         <f>Z35-AA35</f>
-        <v>44130</v>
+        <v>56630</v>
       </c>
       <c r="AC35" s="17" t="str">
         <f>IF(AND($T35=6000, ($T35+$W35-$AB35)&gt;=6000),T35,"")</f>
@@ -4989,10 +4992,10 @@
     </row>
     <row r="36" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>44</v>
@@ -5051,7 +5054,7 @@
         <v>0</v>
       </c>
       <c r="T36" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U36" s="17">
         <v>0</v>
@@ -5070,14 +5073,14 @@
       </c>
       <c r="Z36" s="17">
         <f>SUM(J36:Y36)</f>
-        <v>44130</v>
+        <v>50130</v>
       </c>
       <c r="AA36" s="17">
         <v>0</v>
       </c>
       <c r="AB36" s="14">
         <f>Z36-AA36</f>
-        <v>44130</v>
+        <v>50130</v>
       </c>
       <c r="AC36" s="17" t="str">
         <f>IF(AND($T36=6000, ($T36+$W36-$AB36)&gt;=6000),T36,"")</f>
@@ -5094,16 +5097,16 @@
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>44</v>
       </c>
       <c r="D37" s="16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E37" s="17">
         <v>0</v>
@@ -5126,7 +5129,7 @@
       </c>
       <c r="K37" s="17">
         <f>(1-$D37)*F37</f>
-        <v>26000</v>
+        <v>13000</v>
       </c>
       <c r="L37" s="17">
         <f>G37</f>
@@ -5171,18 +5174,18 @@
         <v>0</v>
       </c>
       <c r="Y37" s="17">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="Z37" s="17">
         <f>SUM(J37:Y37)</f>
-        <v>50630</v>
+        <v>45630</v>
       </c>
       <c r="AA37" s="17">
         <v>0</v>
       </c>
       <c r="AB37" s="14">
         <f>Z37-AA37</f>
-        <v>50630</v>
+        <v>45630</v>
       </c>
       <c r="AC37" s="17" t="str">
         <f>IF(AND($T37=6000, ($T37+$W37-$AB37)&gt;=6000),T37,"")</f>
@@ -5199,13 +5202,13 @@
     </row>
     <row r="38" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>29</v>
+        <v>119</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D38" s="16">
         <v>0.25</v>
@@ -5246,10 +5249,10 @@
         <v>0</v>
       </c>
       <c r="O38" s="17">
-        <v>24870</v>
+        <v>13080</v>
       </c>
       <c r="P38" s="17">
-        <v>10730</v>
+        <v>7550</v>
       </c>
       <c r="Q38" s="17">
         <v>0</v>
@@ -5280,14 +5283,14 @@
       </c>
       <c r="Z38" s="17">
         <f>SUM(J38:Y38)</f>
-        <v>59100</v>
+        <v>44130</v>
       </c>
       <c r="AA38" s="17">
         <v>0</v>
       </c>
       <c r="AB38" s="14">
         <f>Z38-AA38</f>
-        <v>59100</v>
+        <v>44130</v>
       </c>
       <c r="AC38" s="17" t="str">
         <f>IF(AND($T38=6000, ($T38+$W38-$AB38)&gt;=6000),T38,"")</f>
@@ -5304,16 +5307,16 @@
     </row>
     <row r="39" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D39" s="16">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="E39" s="17">
         <v>0</v>
@@ -5336,7 +5339,7 @@
       </c>
       <c r="K39" s="17">
         <f>(1-$D39)*F39</f>
-        <v>13000</v>
+        <v>19500</v>
       </c>
       <c r="L39" s="17">
         <f>G39</f>
@@ -5351,10 +5354,10 @@
         <v>0</v>
       </c>
       <c r="O39" s="17">
-        <v>24870</v>
+        <v>13080</v>
       </c>
       <c r="P39" s="17">
-        <v>10730</v>
+        <v>7550</v>
       </c>
       <c r="Q39" s="17">
         <v>0</v>
@@ -5385,14 +5388,14 @@
       </c>
       <c r="Z39" s="17">
         <f>SUM(J39:Y39)</f>
-        <v>52600</v>
+        <v>44130</v>
       </c>
       <c r="AA39" s="17">
         <v>0</v>
       </c>
       <c r="AB39" s="14">
         <f>Z39-AA39</f>
-        <v>52600</v>
+        <v>44130</v>
       </c>
       <c r="AC39" s="17" t="str">
         <f>IF(AND($T39=6000, ($T39+$W39-$AB39)&gt;=6000),T39,"")</f>
@@ -5409,16 +5412,16 @@
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>40</v>
+        <v>137</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>41</v>
+        <v>138</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D40" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E40" s="17">
         <v>0</v>
@@ -5441,7 +5444,7 @@
       </c>
       <c r="K40" s="17">
         <f>(1-$D40)*F40</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L40" s="17">
         <f>G40</f>
@@ -5456,10 +5459,10 @@
         <v>0</v>
       </c>
       <c r="O40" s="17">
-        <v>24870</v>
+        <v>13080</v>
       </c>
       <c r="P40" s="17">
-        <v>10730</v>
+        <v>7550</v>
       </c>
       <c r="Q40" s="17">
         <v>0</v>
@@ -5490,14 +5493,14 @@
       </c>
       <c r="Z40" s="17">
         <f>SUM(J40:Y40)</f>
-        <v>59100</v>
+        <v>50630</v>
       </c>
       <c r="AA40" s="17">
         <v>0</v>
       </c>
       <c r="AB40" s="14">
         <f>Z40-AA40</f>
-        <v>59100</v>
+        <v>50630</v>
       </c>
       <c r="AC40" s="17" t="str">
         <f>IF(AND($T40=6000, ($T40+$W40-$AB40)&gt;=6000),T40,"")</f>
@@ -5514,10 +5517,10 @@
     </row>
     <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>47</v>
@@ -5576,7 +5579,7 @@
         <v>0</v>
       </c>
       <c r="T41" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U41" s="17">
         <v>0</v>
@@ -5595,14 +5598,14 @@
       </c>
       <c r="Z41" s="17">
         <f>SUM(J41:Y41)</f>
-        <v>65100</v>
+        <v>59100</v>
       </c>
       <c r="AA41" s="17">
         <v>0</v>
       </c>
       <c r="AB41" s="14">
         <f>Z41-AA41</f>
-        <v>65100</v>
+        <v>59100</v>
       </c>
       <c r="AC41" s="17" t="str">
         <f>IF(AND($T41=6000, ($T41+$W41-$AB41)&gt;=6000),T41,"")</f>
@@ -5619,16 +5622,16 @@
     </row>
     <row r="42" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>47</v>
       </c>
       <c r="D42" s="16">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E42" s="17">
         <v>0</v>
@@ -5651,7 +5654,7 @@
       </c>
       <c r="K42" s="17">
         <f>(1-$D42)*F42</f>
-        <v>19500</v>
+        <v>13000</v>
       </c>
       <c r="L42" s="17">
         <f>G42</f>
@@ -5681,7 +5684,7 @@
         <v>0</v>
       </c>
       <c r="T42" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U42" s="17">
         <v>0</v>
@@ -5696,18 +5699,18 @@
         <v>0</v>
       </c>
       <c r="Y42" s="17">
-        <v>18500</v>
+        <v>0</v>
       </c>
       <c r="Z42" s="17">
         <f>SUM(J42:Y42)</f>
-        <v>83600</v>
+        <v>52600</v>
       </c>
       <c r="AA42" s="17">
-        <v>48000</v>
+        <v>0</v>
       </c>
       <c r="AB42" s="14">
         <f>Z42-AA42</f>
-        <v>35600</v>
+        <v>52600</v>
       </c>
       <c r="AC42" s="17" t="str">
         <f>IF(AND($T42=6000, ($T42+$W42-$AB42)&gt;=6000),T42,"")</f>
@@ -5724,10 +5727,10 @@
     </row>
     <row r="43" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
-        <v>88</v>
+        <v>40</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>206</v>
+        <v>41</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>47</v>
@@ -5786,7 +5789,7 @@
         <v>0</v>
       </c>
       <c r="T43" s="17">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="U43" s="17">
         <v>0</v>
@@ -5805,14 +5808,14 @@
       </c>
       <c r="Z43" s="17">
         <f>SUM(J43:Y43)</f>
-        <v>65100</v>
+        <v>59100</v>
       </c>
       <c r="AA43" s="17">
         <v>0</v>
       </c>
       <c r="AB43" s="14">
         <f>Z43-AA43</f>
-        <v>65100</v>
+        <v>59100</v>
       </c>
       <c r="AC43" s="17" t="str">
         <f>IF(AND($T43=6000, ($T43+$W43-$AB43)&gt;=6000),T43,"")</f>
@@ -5829,10 +5832,10 @@
     </row>
     <row r="44" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
-        <v>198</v>
+        <v>60</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>47</v>
@@ -5934,10 +5937,10 @@
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
-        <v>121</v>
+        <v>64</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>47</v>
@@ -6011,18 +6014,18 @@
         <v>0</v>
       </c>
       <c r="Y45" s="17">
-        <v>0</v>
+        <v>18500</v>
       </c>
       <c r="Z45" s="17">
         <f>SUM(J45:Y45)</f>
-        <v>65100</v>
+        <v>83600</v>
       </c>
       <c r="AA45" s="17">
-        <v>0</v>
+        <v>48000</v>
       </c>
       <c r="AB45" s="14">
         <f>Z45-AA45</f>
-        <v>65100</v>
+        <v>35600</v>
       </c>
       <c r="AC45" s="17" t="str">
         <f>IF(AND($T45=6000, ($T45+$W45-$AB45)&gt;=6000),T45,"")</f>
@@ -6039,16 +6042,16 @@
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
-        <v>123</v>
+        <v>88</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>124</v>
+        <v>206</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>47</v>
       </c>
       <c r="D46" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E46" s="17">
         <v>0</v>
@@ -6071,7 +6074,7 @@
       </c>
       <c r="K46" s="17">
         <f>(1-$D46)*F46</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L46" s="17">
         <f>G46</f>
@@ -6116,18 +6119,18 @@
         <v>0</v>
       </c>
       <c r="Y46" s="17">
-        <v>14240</v>
+        <v>0</v>
       </c>
       <c r="Z46" s="17">
         <f>SUM(J46:Y46)</f>
-        <v>85840</v>
+        <v>65100</v>
       </c>
       <c r="AA46" s="17">
         <v>0</v>
       </c>
       <c r="AB46" s="14">
         <f>Z46-AA46</f>
-        <v>85840</v>
+        <v>65100</v>
       </c>
       <c r="AC46" s="17" t="str">
         <f>IF(AND($T46=6000, ($T46+$W46-$AB46)&gt;=6000),T46,"")</f>
@@ -6144,16 +6147,16 @@
     </row>
     <row r="47" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
-        <v>151</v>
+        <v>198</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>152</v>
+        <v>31</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D47" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E47" s="17">
         <v>0</v>
@@ -6165,7 +6168,7 @@
         <v>4000</v>
       </c>
       <c r="H47" s="17">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I47" s="17">
         <v>0</v>
@@ -6176,7 +6179,7 @@
       </c>
       <c r="K47" s="17">
         <f>(1-$D47)*F47</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L47" s="17">
         <f>G47</f>
@@ -6184,29 +6187,29 @@
       </c>
       <c r="M47" s="17">
         <f>(1-$D47)*H47</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N47" s="17">
         <f>(1-$D47)*I47</f>
         <v>0</v>
       </c>
       <c r="O47" s="17">
-        <v>8040</v>
+        <v>24870</v>
       </c>
       <c r="P47" s="17">
-        <v>5300</v>
+        <v>10730</v>
       </c>
       <c r="Q47" s="17">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="R47" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="S47" s="17">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="T47" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U47" s="17">
         <v>0</v>
@@ -6221,18 +6224,18 @@
         <v>0</v>
       </c>
       <c r="Y47" s="17">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="Z47" s="17">
         <f>SUM(J47:Y47)</f>
-        <v>74340</v>
+        <v>65100</v>
       </c>
       <c r="AA47" s="17">
         <v>0</v>
       </c>
       <c r="AB47" s="14">
         <f>Z47-AA47</f>
-        <v>74340</v>
+        <v>65100</v>
       </c>
       <c r="AC47" s="17" t="str">
         <f>IF(AND($T47=6000, ($T47+$W47-$AB47)&gt;=6000),T47,"")</f>
@@ -6249,16 +6252,16 @@
     </row>
     <row r="48" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
-        <v>203</v>
+        <v>121</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>214</v>
+        <v>122</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D48" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E48" s="17">
         <v>0</v>
@@ -6270,7 +6273,7 @@
         <v>4000</v>
       </c>
       <c r="H48" s="17">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I48" s="17">
         <v>0</v>
@@ -6281,7 +6284,7 @@
       </c>
       <c r="K48" s="17">
         <f>(1-$D48)*F48</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L48" s="17">
         <f>G48</f>
@@ -6289,29 +6292,29 @@
       </c>
       <c r="M48" s="17">
         <f>(1-$D48)*H48</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N48" s="17">
         <f>(1-$D48)*I48</f>
         <v>0</v>
       </c>
       <c r="O48" s="17">
-        <v>8040</v>
+        <v>24870</v>
       </c>
       <c r="P48" s="17">
-        <v>5300</v>
+        <v>10730</v>
       </c>
       <c r="Q48" s="17">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="R48" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="S48" s="17">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="T48" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U48" s="17">
         <v>0</v>
@@ -6330,14 +6333,14 @@
       </c>
       <c r="Z48" s="17">
         <f>SUM(J48:Y48)</f>
-        <v>75340</v>
+        <v>65100</v>
       </c>
       <c r="AA48" s="17">
         <v>0</v>
       </c>
       <c r="AB48" s="14">
         <f>Z48-AA48</f>
-        <v>75340</v>
+        <v>65100</v>
       </c>
       <c r="AC48" s="17" t="str">
         <f>IF(AND($T48=6000, ($T48+$W48-$AB48)&gt;=6000),T48,"")</f>
@@ -6354,13 +6357,13 @@
     </row>
     <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
-        <v>188</v>
+        <v>123</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>190</v>
+        <v>124</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D49" s="16">
         <v>0</v>
@@ -6375,7 +6378,7 @@
         <v>4000</v>
       </c>
       <c r="H49" s="17">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I49" s="17">
         <v>0</v>
@@ -6394,29 +6397,29 @@
       </c>
       <c r="M49" s="17">
         <f>(1-$D49)*H49</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N49" s="17">
         <f>(1-$D49)*I49</f>
         <v>0</v>
       </c>
       <c r="O49" s="17">
-        <v>8040</v>
+        <v>24870</v>
       </c>
       <c r="P49" s="17">
-        <v>5300</v>
+        <v>10730</v>
       </c>
       <c r="Q49" s="17">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="R49" s="17">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="S49" s="17">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="T49" s="17">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="U49" s="17">
         <v>0</v>
@@ -6431,18 +6434,18 @@
         <v>0</v>
       </c>
       <c r="Y49" s="17">
-        <v>0</v>
+        <v>14240</v>
       </c>
       <c r="Z49" s="17">
         <f>SUM(J49:Y49)</f>
-        <v>75340</v>
+        <v>85840</v>
       </c>
       <c r="AA49" s="17">
         <v>0</v>
       </c>
       <c r="AB49" s="14">
         <f>Z49-AA49</f>
-        <v>75340</v>
+        <v>85840</v>
       </c>
       <c r="AC49" s="17" t="str">
         <f>IF(AND($T49=6000, ($T49+$W49-$AB49)&gt;=6000),T49,"")</f>
@@ -6459,16 +6462,16 @@
     </row>
     <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>241</v>
+        <v>152</v>
       </c>
       <c r="C50" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D50" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E50" s="17">
         <v>0</v>
@@ -6491,7 +6494,7 @@
       </c>
       <c r="K50" s="17">
         <f>(1-$D50)*F50</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L50" s="17">
         <f>G50</f>
@@ -6499,7 +6502,7 @@
       </c>
       <c r="M50" s="17">
         <f>(1-$D50)*H50</f>
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="N50" s="17">
         <f>(1-$D50)*I50</f>
@@ -6536,18 +6539,18 @@
         <v>0</v>
       </c>
       <c r="Y50" s="17">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="Z50" s="17">
         <f>SUM(J50:Y50)</f>
-        <v>68590</v>
+        <v>74340</v>
       </c>
       <c r="AA50" s="17">
         <v>0</v>
       </c>
       <c r="AB50" s="14">
         <f>Z50-AA50</f>
-        <v>68590</v>
+        <v>74340</v>
       </c>
       <c r="AC50" s="17" t="str">
         <f>IF(AND($T50=6000, ($T50+$W50-$AB50)&gt;=6000),T50,"")</f>
@@ -6564,10 +6567,10 @@
     </row>
     <row r="51" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C51" s="15" t="s">
         <v>49</v>
@@ -6669,10 +6672,10 @@
     </row>
     <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
-        <v>242</v>
+        <v>188</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>50</v>
+        <v>190</v>
       </c>
       <c r="C52" s="15" t="s">
         <v>49</v>
@@ -6774,10 +6777,10 @@
     </row>
     <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>174</v>
+        <v>201</v>
       </c>
       <c r="C53" s="15" t="s">
         <v>49</v>
@@ -6879,10 +6882,10 @@
     </row>
     <row r="54" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>244</v>
+        <v>173</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>245</v>
+        <v>174</v>
       </c>
       <c r="C54" s="15" t="s">
         <v>49</v>
@@ -6984,10 +6987,10 @@
     </row>
     <row r="55" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A55" s="15" t="s">
-        <v>175</v>
+        <v>244</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>176</v>
+        <v>245</v>
       </c>
       <c r="C55" s="15" t="s">
         <v>49</v>
@@ -7061,18 +7064,18 @@
         <v>0</v>
       </c>
       <c r="Y55" s="17">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="Z55" s="17">
         <f>SUM(J55:Y55)</f>
-        <v>77340</v>
+        <v>75340</v>
       </c>
       <c r="AA55" s="17">
         <v>0</v>
       </c>
       <c r="AB55" s="14">
         <f>Z55-AA55</f>
-        <v>77340</v>
+        <v>75340</v>
       </c>
       <c r="AC55" s="17" t="str">
         <f>IF(AND($T55=6000, ($T55+$W55-$AB55)&gt;=6000),T55,"")</f>
@@ -7089,16 +7092,16 @@
     </row>
     <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>213</v>
+        <v>175</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="C56" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D56" s="16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E56" s="17">
         <v>0</v>
@@ -7121,7 +7124,7 @@
       </c>
       <c r="K56" s="17">
         <f>(1-$D56)*F56</f>
-        <v>13000</v>
+        <v>26000</v>
       </c>
       <c r="L56" s="17">
         <f>G56</f>
@@ -7129,7 +7132,7 @@
       </c>
       <c r="M56" s="17">
         <f>(1-$D56)*H56</f>
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="N56" s="17">
         <f>(1-$D56)*I56</f>
@@ -7166,18 +7169,18 @@
         <v>0</v>
       </c>
       <c r="Y56" s="17">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="Z56" s="17">
         <f>SUM(J56:Y56)</f>
-        <v>61840</v>
+        <v>77340</v>
       </c>
       <c r="AA56" s="17">
         <v>0</v>
       </c>
       <c r="AB56" s="14">
         <f>Z56-AA56</f>
-        <v>61840</v>
+        <v>77340</v>
       </c>
       <c r="AC56" s="17" t="str">
         <f>IF(AND($T56=6000, ($T56+$W56-$AB56)&gt;=6000),T56,"")</f>
@@ -7194,16 +7197,16 @@
     </row>
     <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57" s="15" t="s">
-        <v>171</v>
+        <v>213</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
       <c r="C57" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D57" s="16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E57" s="17">
         <v>0</v>
@@ -7226,7 +7229,7 @@
       </c>
       <c r="K57" s="17">
         <f>(1-$D57)*F57</f>
-        <v>26000</v>
+        <v>13000</v>
       </c>
       <c r="L57" s="17">
         <f>G57</f>
@@ -7234,7 +7237,7 @@
       </c>
       <c r="M57" s="17">
         <f>(1-$D57)*H57</f>
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="N57" s="17">
         <f>(1-$D57)*I57</f>
@@ -7275,14 +7278,14 @@
       </c>
       <c r="Z57" s="17">
         <f>SUM(J57:Y57)</f>
-        <v>75340</v>
+        <v>61840</v>
       </c>
       <c r="AA57" s="17">
         <v>0</v>
       </c>
       <c r="AB57" s="14">
         <f>Z57-AA57</f>
-        <v>75340</v>
+        <v>61840</v>
       </c>
       <c r="AC57" s="17" t="str">
         <f>IF(AND($T57=6000, ($T57+$W57-$AB57)&gt;=6000),T57,"")</f>
@@ -7299,16 +7302,16 @@
     </row>
     <row r="58" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
-        <v>88</v>
+        <v>171</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>219</v>
+        <v>172</v>
       </c>
       <c r="C58" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D58" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E58" s="17">
         <v>0</v>
@@ -7331,7 +7334,7 @@
       </c>
       <c r="K58" s="17">
         <f>(1-$D58)*F58</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L58" s="17">
         <f>G58</f>
@@ -7339,7 +7342,7 @@
       </c>
       <c r="M58" s="17">
         <f>(1-$D58)*H58</f>
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="N58" s="17">
         <f>(1-$D58)*I58</f>
@@ -7376,18 +7379,18 @@
         <v>0</v>
       </c>
       <c r="Y58" s="17">
-        <v>-500</v>
+        <v>0</v>
       </c>
       <c r="Z58" s="17">
         <f>SUM(J58:Y58)</f>
-        <v>68090</v>
+        <v>75340</v>
       </c>
       <c r="AA58" s="17">
         <v>0</v>
       </c>
       <c r="AB58" s="14">
         <f>Z58-AA58</f>
-        <v>68090</v>
+        <v>75340</v>
       </c>
       <c r="AC58" s="17" t="str">
         <f>IF(AND($T58=6000, ($T58+$W58-$AB58)&gt;=6000),T58,"")</f>
@@ -7404,10 +7407,10 @@
     </row>
     <row r="59" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
-        <v>159</v>
+        <v>88</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C59" s="15" t="s">
         <v>49</v>
@@ -7481,18 +7484,18 @@
         <v>0</v>
       </c>
       <c r="Y59" s="17">
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="Z59" s="17">
         <f>SUM(J59:Y59)</f>
-        <v>68590</v>
+        <v>68090</v>
       </c>
       <c r="AA59" s="17">
         <v>0</v>
       </c>
       <c r="AB59" s="14">
         <f>Z59-AA59</f>
-        <v>68590</v>
+        <v>68090</v>
       </c>
       <c r="AC59" s="17" t="str">
         <f>IF(AND($T59=6000, ($T59+$W59-$AB59)&gt;=6000),T59,"")</f>
@@ -7509,10 +7512,10 @@
     </row>
     <row r="60" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
-        <v>207</v>
+        <v>159</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C60" s="15" t="s">
         <v>49</v>
@@ -7586,18 +7589,18 @@
         <v>0</v>
       </c>
       <c r="Y60" s="17">
-        <v>19200</v>
+        <v>0</v>
       </c>
       <c r="Z60" s="17">
         <f>SUM(J60:Y60)</f>
-        <v>87790</v>
+        <v>68590</v>
       </c>
       <c r="AA60" s="17">
         <v>0</v>
       </c>
       <c r="AB60" s="14">
         <f>Z60-AA60</f>
-        <v>87790</v>
+        <v>68590</v>
       </c>
       <c r="AC60" s="17" t="str">
         <f>IF(AND($T60=6000, ($T60+$W60-$AB60)&gt;=6000),T60,"")</f>
@@ -7617,7 +7620,7 @@
         <v>207</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C61" s="15" t="s">
         <v>49</v>
@@ -7719,10 +7722,10 @@
     </row>
     <row r="62" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
-        <v>98</v>
+        <v>207</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>145</v>
+        <v>216</v>
       </c>
       <c r="C62" s="15" t="s">
         <v>49</v>
@@ -7796,18 +7799,18 @@
         <v>0</v>
       </c>
       <c r="Y62" s="17">
-        <v>0</v>
+        <v>19200</v>
       </c>
       <c r="Z62" s="17">
         <f>SUM(J62:Y62)</f>
-        <v>68590</v>
+        <v>87790</v>
       </c>
       <c r="AA62" s="17">
         <v>0</v>
       </c>
       <c r="AB62" s="14">
         <f>Z62-AA62</f>
-        <v>68590</v>
+        <v>87790</v>
       </c>
       <c r="AC62" s="17" t="str">
         <f>IF(AND($T62=6000, ($T62+$W62-$AB62)&gt;=6000),T62,"")</f>
@@ -7824,10 +7827,10 @@
     </row>
     <row r="63" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
-        <v>204</v>
+        <v>98</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>205</v>
+        <v>145</v>
       </c>
       <c r="C63" s="15" t="s">
         <v>49</v>
@@ -7901,18 +7904,18 @@
         <v>0</v>
       </c>
       <c r="Y63" s="17">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="Z63" s="17">
         <f>SUM(J63:Y63)</f>
-        <v>72090</v>
+        <v>68590</v>
       </c>
       <c r="AA63" s="17">
         <v>0</v>
       </c>
       <c r="AB63" s="14">
         <f>Z63-AA63</f>
-        <v>72090</v>
+        <v>68590</v>
       </c>
       <c r="AC63" s="17" t="str">
         <f>IF(AND($T63=6000, ($T63+$W63-$AB63)&gt;=6000),T63,"")</f>
@@ -7929,16 +7932,16 @@
     </row>
     <row r="64" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C64" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D64" s="16">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E64" s="17">
         <v>0</v>
@@ -7961,7 +7964,7 @@
       </c>
       <c r="K64" s="17">
         <f>(1-$D64)*F64</f>
-        <v>26000</v>
+        <v>19500</v>
       </c>
       <c r="L64" s="17">
         <f>G64</f>
@@ -7969,7 +7972,7 @@
       </c>
       <c r="M64" s="17">
         <f>(1-$D64)*H64</f>
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="N64" s="17">
         <f>(1-$D64)*I64</f>
@@ -8006,18 +8009,18 @@
         <v>0</v>
       </c>
       <c r="Y64" s="17">
-        <v>-10000</v>
+        <v>3500</v>
       </c>
       <c r="Z64" s="17">
         <f>SUM(J64:Y64)</f>
-        <v>65340</v>
+        <v>72090</v>
       </c>
       <c r="AA64" s="17">
         <v>0</v>
       </c>
       <c r="AB64" s="14">
         <f>Z64-AA64</f>
-        <v>65340</v>
+        <v>72090</v>
       </c>
       <c r="AC64" s="17" t="str">
         <f>IF(AND($T64=6000, ($T64+$W64-$AB64)&gt;=6000),T64,"")</f>
@@ -8034,16 +8037,16 @@
     </row>
     <row r="65" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A65" s="15" t="s">
-        <v>121</v>
+        <v>211</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>243</v>
+        <v>212</v>
       </c>
       <c r="C65" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D65" s="16">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E65" s="17">
         <v>0</v>
@@ -8066,7 +8069,7 @@
       </c>
       <c r="K65" s="17">
         <f>(1-$D65)*F65</f>
-        <v>19500</v>
+        <v>26000</v>
       </c>
       <c r="L65" s="17">
         <f>G65</f>
@@ -8074,7 +8077,7 @@
       </c>
       <c r="M65" s="17">
         <f>(1-$D65)*H65</f>
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="N65" s="17">
         <f>(1-$D65)*I65</f>
@@ -8111,18 +8114,18 @@
         <v>0</v>
       </c>
       <c r="Y65" s="17">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="Z65" s="17">
         <f>SUM(J65:Y65)</f>
-        <v>68590</v>
+        <v>65340</v>
       </c>
       <c r="AA65" s="17">
         <v>0</v>
       </c>
       <c r="AB65" s="14">
         <f>Z65-AA65</f>
-        <v>68590</v>
+        <v>65340</v>
       </c>
       <c r="AC65" s="17" t="str">
         <f>IF(AND($T65=6000, ($T65+$W65-$AB65)&gt;=6000),T65,"")</f>
@@ -13943,7 +13946,7 @@
       </c>
       <c r="Z121" s="29">
         <f>SUM(Z2:Z120)</f>
-        <v>7931310</v>
+        <v>7807440</v>
       </c>
       <c r="AA121" s="29">
         <f>SUM(AA2:AA120)</f>
@@ -13951,7 +13954,7 @@
       </c>
       <c r="AB121" s="29">
         <f>SUM(AB2:AB120)</f>
-        <v>7883310</v>
+        <v>7759440</v>
       </c>
       <c r="AC121" s="29">
         <f>SUM(AC2:AC120)</f>

</xml_diff>

<commit_message>
Update generated data & student payment
Regenerated data to reflect a recorded payment. Updated docs/data/meta.json (generatedAt; currentOutstanding 7,203,495 -> 7,160,495). Updated docs/data/students.json for a student: latestBalance 44,280 -> 1,280 and term record updated (total 44,280, paid 43,000, balance 1,280). Replaced source/2026 - 2027 FEE.xlsx with the updated binary.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/source/2026 - 2027 FEE.xlsx
+++ b/source/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A16758B-C668-4C10-8774-B70E2515AE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056D1BA0-9702-4A36-843B-44663388CA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="256">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -800,6 +800,12 @@
   <si>
     <t>CRECHE</t>
   </si>
+  <si>
+    <t>NIP:PAUL SUNDAY ADEDOJA</t>
+  </si>
+  <si>
+    <t>ADEDOJA FAMILY</t>
+  </si>
 </sst>
 </file>
 
@@ -8750,11 +8756,11 @@
         <v>44280</v>
       </c>
       <c r="AA71" s="24">
-        <v>0</v>
+        <v>43000</v>
       </c>
       <c r="AB71" s="20">
         <f>Z71-AA71</f>
-        <v>44280</v>
+        <v>1280</v>
       </c>
       <c r="AC71" s="24" t="str">
         <f>IF(AND($T71=6000, ($T71+$W71-$AB71)&gt;=6000),T71,"")</f>
@@ -13949,11 +13955,11 @@
       </c>
       <c r="AA121" s="27">
         <f>SUM(AA2:AA120)</f>
-        <v>48000</v>
+        <v>91000</v>
       </c>
       <c r="AB121" s="27">
         <f>SUM(AB2:AB120)</f>
-        <v>7203495</v>
+        <v>7160495</v>
       </c>
       <c r="AC121" s="27">
         <f>SUM(AC2:AC120)</f>
@@ -22239,7 +22245,23 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>46255</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="9">
+        <v>43000</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
     <row r="4" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>